<commit_message>
Rep D dry weights
</commit_message>
<xml_diff>
--- a/data_in/TF-GH-Datasheets.xlsx
+++ b/data_in/TF-GH-Datasheets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacksonstrand/Documents/GitHub/toadflax_phys_2026/data_in/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26E97301-8D6B-D94A-BF76-0E4BB3E79102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10707D24-F402-ED42-895F-723D3A6417D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4080" yWindow="1600" windowWidth="30240" windowHeight="18980" firstSheet="3" activeTab="17" xr2:uid="{68B39474-F999-644F-96EB-FFA9F0452C84}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" firstSheet="6" activeTab="21" xr2:uid="{68B39474-F999-644F-96EB-FFA9F0452C84}"/>
   </bookViews>
   <sheets>
     <sheet name="Awk7" sheetId="12" r:id="rId1"/>
@@ -33,6 +33,8 @@
     <sheet name="Dwk10" sheetId="18" r:id="rId18"/>
     <sheet name="Fwk7" sheetId="19" r:id="rId19"/>
     <sheet name="Gwk7" sheetId="20" r:id="rId20"/>
+    <sheet name="Ewk10" sheetId="21" r:id="rId21"/>
+    <sheet name="Hwk7" sheetId="22" r:id="rId22"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -55,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="245">
   <si>
     <t>sample</t>
   </si>
@@ -763,6 +765,33 @@
   </si>
   <si>
     <t>5 small galls above high leaf</t>
+  </si>
+  <si>
+    <t>1 gall between lower and upper</t>
+  </si>
+  <si>
+    <t>some thrips leaf damage</t>
+  </si>
+  <si>
+    <t>heavily stunted, full of galls</t>
+  </si>
+  <si>
+    <t>several pseudogalls near top of stem</t>
+  </si>
+  <si>
+    <t>5 small galls between mid and high</t>
+  </si>
+  <si>
+    <t>1 gall between low and high, 3 above high</t>
+  </si>
+  <si>
+    <t>some thrips damage on leaves</t>
+  </si>
+  <si>
+    <t>original stem stunted, but other larger stems exist on plant</t>
+  </si>
+  <si>
+    <t>1 gall between low and mid, the rest on secondaries</t>
   </si>
 </sst>
 </file>
@@ -4724,6 +4753,543 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA1BCF96-1CA2-AA43-8090-EA52E48E288B}">
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B3" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B4" s="1">
+        <v>0.40833333333333333</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5" s="1">
+        <v>0.42499999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C6" t="s">
+        <v>227</v>
+      </c>
+      <c r="D6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E6" t="s">
+        <v>117</v>
+      </c>
+      <c r="F6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="D7">
+        <v>23.1</v>
+      </c>
+      <c r="E7">
+        <v>42.7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>5.5</v>
+      </c>
+      <c r="D8">
+        <v>32.1</v>
+      </c>
+      <c r="E8">
+        <v>56.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9">
+        <v>3.2</v>
+      </c>
+      <c r="D9">
+        <v>20.8</v>
+      </c>
+      <c r="E9">
+        <v>41.2</v>
+      </c>
+      <c r="F9" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10">
+        <v>6.8</v>
+      </c>
+      <c r="D10">
+        <v>31.2</v>
+      </c>
+      <c r="E10">
+        <v>58.3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11">
+        <v>5.4</v>
+      </c>
+      <c r="D11">
+        <v>26.9</v>
+      </c>
+      <c r="E11">
+        <v>57.2</v>
+      </c>
+      <c r="F11" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12">
+        <v>2.9</v>
+      </c>
+      <c r="D12">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="E12">
+        <v>10.3</v>
+      </c>
+      <c r="F12" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13">
+        <v>7.3</v>
+      </c>
+      <c r="D13">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="E13">
+        <v>49.1</v>
+      </c>
+      <c r="F13" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="D14">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="E14">
+        <v>42.6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15">
+        <v>5</v>
+      </c>
+      <c r="D15">
+        <v>28</v>
+      </c>
+      <c r="E15">
+        <v>52.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16">
+        <v>3.4</v>
+      </c>
+      <c r="D16">
+        <v>16.600000000000001</v>
+      </c>
+      <c r="E16">
+        <v>34.1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="D17">
+        <v>11.1</v>
+      </c>
+      <c r="E17">
+        <v>33.6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18">
+        <v>5.2</v>
+      </c>
+      <c r="D18">
+        <v>25.1</v>
+      </c>
+      <c r="E18">
+        <v>47.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8024103-CD47-F94D-9CDE-2FEBA51A685A}">
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B3" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B4" s="1">
+        <v>0.42708333333333331</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5" s="1">
+        <v>0.44930555555555557</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C6" t="s">
+        <v>227</v>
+      </c>
+      <c r="D6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E6" t="s">
+        <v>117</v>
+      </c>
+      <c r="F6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7">
+        <v>6.7</v>
+      </c>
+      <c r="C7">
+        <v>15.4</v>
+      </c>
+      <c r="D7">
+        <v>22.2</v>
+      </c>
+      <c r="E7">
+        <v>29.4</v>
+      </c>
+      <c r="F7" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>6.8</v>
+      </c>
+      <c r="C8">
+        <v>16.7</v>
+      </c>
+      <c r="D8">
+        <v>39</v>
+      </c>
+      <c r="E8">
+        <v>57.7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9">
+        <v>7.2</v>
+      </c>
+      <c r="D9">
+        <v>15.2</v>
+      </c>
+      <c r="E9">
+        <v>30.3</v>
+      </c>
+      <c r="F9" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
+      <c r="C10">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="D10">
+        <v>24.7</v>
+      </c>
+      <c r="E10">
+        <v>43.8</v>
+      </c>
+      <c r="F10" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="C11">
+        <v>7.2</v>
+      </c>
+      <c r="D11">
+        <v>13.6</v>
+      </c>
+      <c r="E11">
+        <v>21.6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>3.4</v>
+      </c>
+      <c r="C12">
+        <v>6.6</v>
+      </c>
+      <c r="D12">
+        <v>21.1</v>
+      </c>
+      <c r="E12">
+        <v>33.1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13">
+        <v>12.3</v>
+      </c>
+      <c r="D13">
+        <v>19.100000000000001</v>
+      </c>
+      <c r="E13">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14">
+        <v>5.7</v>
+      </c>
+      <c r="C14">
+        <v>14.8</v>
+      </c>
+      <c r="D14">
+        <v>18.5</v>
+      </c>
+      <c r="E14">
+        <v>56.9</v>
+      </c>
+      <c r="F14" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="D15">
+        <v>10.1</v>
+      </c>
+      <c r="E15">
+        <v>12.8</v>
+      </c>
+      <c r="F15" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="C16">
+        <v>7.6</v>
+      </c>
+      <c r="D16">
+        <v>15</v>
+      </c>
+      <c r="E16">
+        <v>26.6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17">
+        <v>10.5</v>
+      </c>
+      <c r="C17">
+        <v>19.899999999999999</v>
+      </c>
+      <c r="D17">
+        <v>38</v>
+      </c>
+      <c r="E17">
+        <v>57.3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>6.6</v>
+      </c>
+      <c r="C18">
+        <v>10.8</v>
+      </c>
+      <c r="D18">
+        <v>20</v>
+      </c>
+      <c r="E18">
+        <v>26.9</v>
+      </c>
+      <c r="F18" t="s">
+        <v>244</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65038CB4-CCB8-1844-B40B-D1E84A08D825}">
   <dimension ref="A1:G15"/>

</xml_diff>

<commit_message>
Rep F Wk 10 GH data
</commit_message>
<xml_diff>
--- a/data_in/TF-GH-Datasheets.xlsx
+++ b/data_in/TF-GH-Datasheets.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacksonstrand/Documents/GitHub/toadflax_phys_2026/data_in/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10707D24-F402-ED42-895F-723D3A6417D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26D1131D-55E6-7447-8E92-1D610BE5DA44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" firstSheet="6" activeTab="21" xr2:uid="{68B39474-F999-644F-96EB-FFA9F0452C84}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" firstSheet="6" activeTab="22" xr2:uid="{68B39474-F999-644F-96EB-FFA9F0452C84}"/>
   </bookViews>
   <sheets>
     <sheet name="Awk7" sheetId="12" r:id="rId1"/>
@@ -35,6 +35,7 @@
     <sheet name="Gwk7" sheetId="20" r:id="rId20"/>
     <sheet name="Ewk10" sheetId="21" r:id="rId21"/>
     <sheet name="Hwk7" sheetId="22" r:id="rId22"/>
+    <sheet name="Fwk10" sheetId="23" r:id="rId23"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -57,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="252">
   <si>
     <t>sample</t>
   </si>
@@ -792,6 +793,27 @@
   </si>
   <si>
     <t>1 gall between low and mid, the rest on secondaries</t>
+  </si>
+  <si>
+    <t>aphids in flowers</t>
+  </si>
+  <si>
+    <t>some thrips scarring</t>
+  </si>
+  <si>
+    <t>2 galls between lower and upper, 2 above upper</t>
+  </si>
+  <si>
+    <t>2 galls between mid and upper 3 above upper</t>
+  </si>
+  <si>
+    <t>lots of sawdust/frass</t>
+  </si>
+  <si>
+    <t>several lumps between lower and upper, one gall right at upper, 1 above upper</t>
+  </si>
+  <si>
+    <t>1 gall near top of stem</t>
   </si>
 </sst>
 </file>
@@ -5287,6 +5309,272 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE396B39-5FD4-7140-A9BA-0CD8419CABFD}">
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B3" s="2">
+        <v>46141</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B4" s="1">
+        <v>0.3888888888888889</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5" s="1">
+        <v>0.40625</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C6" t="s">
+        <v>227</v>
+      </c>
+      <c r="D6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E6" t="s">
+        <v>117</v>
+      </c>
+      <c r="F6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7">
+        <v>9.4</v>
+      </c>
+      <c r="D7">
+        <v>18.899999999999999</v>
+      </c>
+      <c r="E7">
+        <v>52.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>12.7</v>
+      </c>
+      <c r="D8">
+        <v>21.5</v>
+      </c>
+      <c r="E8">
+        <v>53.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9">
+        <v>8.5</v>
+      </c>
+      <c r="D9">
+        <v>15.1</v>
+      </c>
+      <c r="E9">
+        <v>56.4</v>
+      </c>
+      <c r="F9" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10">
+        <v>9.1</v>
+      </c>
+      <c r="D10">
+        <v>15.8</v>
+      </c>
+      <c r="E10">
+        <v>48.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11">
+        <v>6.9</v>
+      </c>
+      <c r="D11">
+        <v>14.3</v>
+      </c>
+      <c r="E11">
+        <v>55.5</v>
+      </c>
+      <c r="F11" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12">
+        <v>8.5</v>
+      </c>
+      <c r="D12">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="E12">
+        <v>45.9</v>
+      </c>
+      <c r="F12" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="D13">
+        <v>22.2</v>
+      </c>
+      <c r="E13">
+        <v>55.4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14">
+        <v>11.7</v>
+      </c>
+      <c r="D14">
+        <v>19.399999999999999</v>
+      </c>
+      <c r="E14">
+        <v>51.7</v>
+      </c>
+      <c r="F14" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15">
+        <v>4.5</v>
+      </c>
+      <c r="C15">
+        <v>11.1</v>
+      </c>
+      <c r="D15">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="E15">
+        <v>40.1</v>
+      </c>
+      <c r="F15" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16">
+        <v>5.2</v>
+      </c>
+      <c r="D16">
+        <v>12.5</v>
+      </c>
+      <c r="E16">
+        <v>29.4</v>
+      </c>
+      <c r="F16" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="D17">
+        <v>20.2</v>
+      </c>
+      <c r="E17">
+        <v>54.3</v>
+      </c>
+      <c r="F17" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>10.1</v>
+      </c>
+      <c r="D18">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="E18">
+        <v>55.4</v>
+      </c>
+      <c r="F18" t="s">
+        <v>251</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>